<commit_message>
Publish dual analysis (Clean vs All-Data) and Day-of-Week Bus Speed chart
</commit_message>
<xml_diff>
--- a/output/conclusion/summary_tables/Kolkata_Metro_vs_Bus_Commuter_Mastery.xlsx
+++ b/output/conclusion/summary_tables/Kolkata_Metro_vs_Bus_Commuter_Mastery.xlsx
@@ -9,13 +9,15 @@
     <sheet sheetId="3" name="🚌 Individual Bus Dynamics" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="🚇 Individual Metro Dynamics" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="⚔️ Head-to-Head Rankings" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="⚖️ Clean vs All-Data Contrast" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="📅 Bus Speed by Day of Week" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="420">
   <si>
     <t>KOLKATA METRO vs SURFACE BUS: MULTIMODAL COMMUTE MASTERY</t>
   </si>
@@ -1038,13 +1040,250 @@
   </si>
   <si>
     <t>+-4.6 min</t>
+  </si>
+  <si>
+    <t>DUAL ANALYSIS CONTRAST: CLEAN (CORRECT) DATASET vs ALL RAW DATA</t>
+  </si>
+  <si>
+    <t>METRIC / EVALUATION DIMENSION</t>
+  </si>
+  <si>
+    <t>ANALYSIS A: CLEAN DATA (100% Correct)</t>
+  </si>
+  <si>
+    <t>ANALYSIS B: ALL RAW DATA (With Anomalies)</t>
+  </si>
+  <si>
+    <t>IMPACT / DISTORTION</t>
+  </si>
+  <si>
+    <t>METHODOLOGICAL RATIONALE</t>
+  </si>
+  <si>
+    <t>Total Sample Size (N)</t>
+  </si>
+  <si>
+    <t>1,952 observations</t>
+  </si>
+  <si>
+    <t>2,300 observations</t>
+  </si>
+  <si>
+    <t>-348 anomalous runs removed</t>
+  </si>
+  <si>
+    <t>Anomalous walking fallbacks &amp; closed Sundays excluded</t>
+  </si>
+  <si>
+    <t>Metro Win Rate vs Bus</t>
+  </si>
+  <si>
+    <t>99.0% (1,932 wins)</t>
+  </si>
+  <si>
+    <t>84.4% (1,941 wins)</t>
+  </si>
+  <si>
+    <t>-14.6% artificial penalty</t>
+  </si>
+  <si>
+    <t>In raw data, bus falsely "won" against pedestrians walking along NH 12</t>
+  </si>
+  <si>
+    <t>Bus Win Rate vs Metro</t>
+  </si>
+  <si>
+    <t>1.0% (20 wins)</t>
+  </si>
+  <si>
+    <t>15.6% (359 wins)</t>
+  </si>
+  <si>
+    <t>+14.6% artificial inflation</t>
+  </si>
+  <si>
+    <t>Raw data counts midday closures as bus "victories"</t>
+  </si>
+  <si>
+    <t>Metro Mean Travel Time</t>
+  </si>
+  <si>
+    <t>16.6 min</t>
+  </si>
+  <si>
+    <t>18.6 min</t>
+  </si>
+  <si>
+    <t>+2.0 min artificial delay</t>
+  </si>
+  <si>
+    <t>Walking 57 mins on Purple Line falsely pulls metro average up</t>
+  </si>
+  <si>
+    <t>Metro Std Deviation (σ)</t>
+  </si>
+  <si>
+    <t>±7.4 min</t>
+  </si>
+  <si>
+    <t>±10.8 min</t>
+  </si>
+  <si>
+    <t>+46% artificial variance</t>
+  </si>
+  <si>
+    <t>Real metro trains have σ &lt; 1 min; walking routes inject artificial chaos</t>
+  </si>
+  <si>
+    <t>Bus Mean Travel Time</t>
+  </si>
+  <si>
+    <t>28.0 min</t>
+  </si>
+  <si>
+    <t>27.2 min</t>
+  </si>
+  <si>
+    <t>-0.8 min shift</t>
+  </si>
+  <si>
+    <t>Bus service remained consistent across both datasets</t>
+  </si>
+  <si>
+    <t>Average Time Saved by Metro</t>
+  </si>
+  <si>
+    <t>+11.4 min / trip</t>
+  </si>
+  <si>
+    <t>+8.6 min / trip</t>
+  </si>
+  <si>
+    <t>-2.8 min / trip depressed</t>
+  </si>
+  <si>
+    <t>Clean data shows the true operational advantage of Metro</t>
+  </si>
+  <si>
+    <t>Purple Line Win Rate</t>
+  </si>
+  <si>
+    <t>82.0% (Clean Active Trains)</t>
+  </si>
+  <si>
+    <t>41.2% (Raw Unfiltered)</t>
+  </si>
+  <si>
+    <t>-40.8% catastrophic distortion</t>
+  </si>
+  <si>
+    <t>Midday shuttle pause resulted in 108 walking fallbacks on Purple Line</t>
+  </si>
+  <si>
+    <t>Line Alignment</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+  <si>
+    <t>Mon (km/h)</t>
+  </si>
+  <si>
+    <t>Tue (km/h)</t>
+  </si>
+  <si>
+    <t>Wed (km/h)</t>
+  </si>
+  <si>
+    <t>Thu (km/h)</t>
+  </si>
+  <si>
+    <t>Fri (km/h)</t>
+  </si>
+  <si>
+    <t>Sat (km/h)</t>
+  </si>
+  <si>
+    <t>Sun (km/h)</t>
+  </si>
+  <si>
+    <t>7-Day Avg (km/h)</t>
+  </si>
+  <si>
+    <t>13.2 km</t>
+  </si>
+  <si>
+    <t>15.1 km</t>
+  </si>
+  <si>
+    <t>4 km</t>
+  </si>
+  <si>
+    <t>6.1 km</t>
+  </si>
+  <si>
+    <t>6.6 km</t>
+  </si>
+  <si>
+    <t>10 km</t>
+  </si>
+  <si>
+    <t>7.5 km</t>
+  </si>
+  <si>
+    <t>10.1 km</t>
+  </si>
+  <si>
+    <t>11.7 km</t>
+  </si>
+  <si>
+    <t>8 km</t>
+  </si>
+  <si>
+    <t>5.5 km</t>
+  </si>
+  <si>
+    <t>5.4 km</t>
+  </si>
+  <si>
+    <t>6.7 km</t>
+  </si>
+  <si>
+    <t>10.8 km</t>
+  </si>
+  <si>
+    <t>11.5 km</t>
+  </si>
+  <si>
+    <t>5.2 km</t>
+  </si>
+  <si>
+    <t>10.5 km</t>
+  </si>
+  <si>
+    <t>4.8 km</t>
+  </si>
+  <si>
+    <t>5.3 km</t>
+  </si>
+  <si>
+    <t>8.4 km</t>
+  </si>
+  <si>
+    <t>3.1 km</t>
+  </si>
+  <si>
+    <t>1.7 km</t>
+  </si>
+  <si>
+    <t>3.7 km</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1103,6 +1342,16 @@
       <b/>
       <color rgb="FFD96B27"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFC00000"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -1154,7 +1403,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1183,6 +1432,12 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1775,7 +2030,7 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3253,7 +3508,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4104,7 +4359,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4877,7 +5132,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5651,6 +5906,1378 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:F12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="4" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="32" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+    </row>
+    <row r="4" spans="1:6" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>342</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>343</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>348</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>349</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>353</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>354</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>358</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>359</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>363</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>364</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>368</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>369</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>374</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>378</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>379</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>383</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>386</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N26"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="3" width="22" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:14" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>387</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>388</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>389</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>390</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>391</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="L1" s="14" t="s">
+        <v>394</v>
+      </c>
+      <c r="M1" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" t="s">
+        <v>397</v>
+      </c>
+      <c r="G2">
+        <v>14.8</v>
+      </c>
+      <c r="H2">
+        <v>14.5</v>
+      </c>
+      <c r="I2">
+        <v>14.7</v>
+      </c>
+      <c r="J2">
+        <v>14.7</v>
+      </c>
+      <c r="K2">
+        <v>14.7</v>
+      </c>
+      <c r="L2">
+        <v>14.7</v>
+      </c>
+      <c r="M2">
+        <v>14.5</v>
+      </c>
+      <c r="N2" s="21">
+        <v>14.7</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" t="s">
+        <v>398</v>
+      </c>
+      <c r="G3">
+        <v>17.8</v>
+      </c>
+      <c r="H3">
+        <v>17.8</v>
+      </c>
+      <c r="I3">
+        <v>17.8</v>
+      </c>
+      <c r="J3">
+        <v>17.8</v>
+      </c>
+      <c r="K3">
+        <v>17.8</v>
+      </c>
+      <c r="L3">
+        <v>17.8</v>
+      </c>
+      <c r="M3">
+        <v>17.8</v>
+      </c>
+      <c r="N3">
+        <v>17.8</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" t="s">
+        <v>399</v>
+      </c>
+      <c r="G4">
+        <v>16.2</v>
+      </c>
+      <c r="H4">
+        <v>15.6</v>
+      </c>
+      <c r="I4">
+        <v>15.2</v>
+      </c>
+      <c r="J4">
+        <v>16.7</v>
+      </c>
+      <c r="K4">
+        <v>16.7</v>
+      </c>
+      <c r="L4">
+        <v>16.4</v>
+      </c>
+      <c r="M4">
+        <v>17</v>
+      </c>
+      <c r="N4">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F5" t="s">
+        <v>400</v>
+      </c>
+      <c r="G5">
+        <v>18.8</v>
+      </c>
+      <c r="H5">
+        <v>18.4</v>
+      </c>
+      <c r="I5">
+        <v>18.4</v>
+      </c>
+      <c r="J5">
+        <v>17.7</v>
+      </c>
+      <c r="K5">
+        <v>17.7</v>
+      </c>
+      <c r="L5">
+        <v>18.4</v>
+      </c>
+      <c r="M5">
+        <v>18.5</v>
+      </c>
+      <c r="N5">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" t="s">
+        <v>401</v>
+      </c>
+      <c r="G6">
+        <v>22</v>
+      </c>
+      <c r="H6">
+        <v>22</v>
+      </c>
+      <c r="I6">
+        <v>22</v>
+      </c>
+      <c r="J6">
+        <v>22</v>
+      </c>
+      <c r="K6">
+        <v>22</v>
+      </c>
+      <c r="L6">
+        <v>22</v>
+      </c>
+      <c r="M6">
+        <v>22</v>
+      </c>
+      <c r="N6" s="20">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F7" t="s">
+        <v>400</v>
+      </c>
+      <c r="G7">
+        <v>15.2</v>
+      </c>
+      <c r="H7">
+        <v>14.5</v>
+      </c>
+      <c r="I7">
+        <v>15.2</v>
+      </c>
+      <c r="J7">
+        <v>14.4</v>
+      </c>
+      <c r="K7">
+        <v>14.4</v>
+      </c>
+      <c r="L7">
+        <v>15.2</v>
+      </c>
+      <c r="M7">
+        <v>14.5</v>
+      </c>
+      <c r="N7" s="21">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s">
+        <v>402</v>
+      </c>
+      <c r="G8">
+        <v>20.1</v>
+      </c>
+      <c r="H8">
+        <v>20.2</v>
+      </c>
+      <c r="I8">
+        <v>20</v>
+      </c>
+      <c r="J8">
+        <v>20</v>
+      </c>
+      <c r="K8">
+        <v>20</v>
+      </c>
+      <c r="L8">
+        <v>20</v>
+      </c>
+      <c r="M8">
+        <v>19.8</v>
+      </c>
+      <c r="N8" s="20">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" t="s">
+        <v>403</v>
+      </c>
+      <c r="G9">
+        <v>20.5</v>
+      </c>
+      <c r="H9">
+        <v>20.5</v>
+      </c>
+      <c r="I9">
+        <v>20.5</v>
+      </c>
+      <c r="J9">
+        <v>20.5</v>
+      </c>
+      <c r="K9">
+        <v>20.5</v>
+      </c>
+      <c r="L9">
+        <v>20.5</v>
+      </c>
+      <c r="M9">
+        <v>20.5</v>
+      </c>
+      <c r="N9" s="20">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F10" t="s">
+        <v>404</v>
+      </c>
+      <c r="G10">
+        <v>16.7</v>
+      </c>
+      <c r="H10">
+        <v>16.2</v>
+      </c>
+      <c r="I10">
+        <v>16.1</v>
+      </c>
+      <c r="J10">
+        <v>16.2</v>
+      </c>
+      <c r="K10">
+        <v>16.2</v>
+      </c>
+      <c r="L10">
+        <v>16</v>
+      </c>
+      <c r="M10">
+        <v>16.2</v>
+      </c>
+      <c r="N10">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" t="s">
+        <v>405</v>
+      </c>
+      <c r="G11">
+        <v>17.4</v>
+      </c>
+      <c r="H11">
+        <v>17.4</v>
+      </c>
+      <c r="I11">
+        <v>17.4</v>
+      </c>
+      <c r="J11">
+        <v>17.3</v>
+      </c>
+      <c r="K11">
+        <v>17.3</v>
+      </c>
+      <c r="L11">
+        <v>17.4</v>
+      </c>
+      <c r="M11">
+        <v>17.3</v>
+      </c>
+      <c r="N11">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>125</v>
+      </c>
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" t="s">
+        <v>406</v>
+      </c>
+      <c r="G12">
+        <v>18.9</v>
+      </c>
+      <c r="H12">
+        <v>19</v>
+      </c>
+      <c r="I12">
+        <v>18.9</v>
+      </c>
+      <c r="J12">
+        <v>19</v>
+      </c>
+      <c r="K12">
+        <v>18.9</v>
+      </c>
+      <c r="L12">
+        <v>19</v>
+      </c>
+      <c r="M12">
+        <v>18.9</v>
+      </c>
+      <c r="N12">
+        <v>18.9</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" t="s">
+        <v>96</v>
+      </c>
+      <c r="C13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" t="s">
+        <v>407</v>
+      </c>
+      <c r="G13">
+        <v>17.6</v>
+      </c>
+      <c r="H13">
+        <v>17.7</v>
+      </c>
+      <c r="I13">
+        <v>17.6</v>
+      </c>
+      <c r="J13">
+        <v>17.6</v>
+      </c>
+      <c r="K13">
+        <v>17.6</v>
+      </c>
+      <c r="L13">
+        <v>17.6</v>
+      </c>
+      <c r="M13">
+        <v>17.7</v>
+      </c>
+      <c r="N13">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" t="s">
+        <v>95</v>
+      </c>
+      <c r="E14" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" t="s">
+        <v>408</v>
+      </c>
+      <c r="G14">
+        <v>12.3</v>
+      </c>
+      <c r="H14">
+        <v>12.3</v>
+      </c>
+      <c r="I14">
+        <v>12.6</v>
+      </c>
+      <c r="J14">
+        <v>12.3</v>
+      </c>
+      <c r="K14">
+        <v>12.5</v>
+      </c>
+      <c r="L14">
+        <v>12.2</v>
+      </c>
+      <c r="M14">
+        <v>12.7</v>
+      </c>
+      <c r="N14" s="21">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" t="s">
+        <v>96</v>
+      </c>
+      <c r="C15" t="s">
+        <v>97</v>
+      </c>
+      <c r="D15" t="s">
+        <v>95</v>
+      </c>
+      <c r="E15" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" t="s">
+        <v>409</v>
+      </c>
+      <c r="G15">
+        <v>15.8</v>
+      </c>
+      <c r="H15">
+        <v>15.7</v>
+      </c>
+      <c r="I15">
+        <v>15.7</v>
+      </c>
+      <c r="J15">
+        <v>15.7</v>
+      </c>
+      <c r="K15">
+        <v>15.7</v>
+      </c>
+      <c r="L15">
+        <v>15.7</v>
+      </c>
+      <c r="M15">
+        <v>15.6</v>
+      </c>
+      <c r="N15" s="21">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" t="s">
+        <v>98</v>
+      </c>
+      <c r="F16" t="s">
+        <v>410</v>
+      </c>
+      <c r="G16">
+        <v>19.1</v>
+      </c>
+      <c r="H16">
+        <v>19.1</v>
+      </c>
+      <c r="I16">
+        <v>19.1</v>
+      </c>
+      <c r="J16">
+        <v>19.1</v>
+      </c>
+      <c r="K16">
+        <v>19.1</v>
+      </c>
+      <c r="L16">
+        <v>19.1</v>
+      </c>
+      <c r="M16">
+        <v>19.1</v>
+      </c>
+      <c r="N16">
+        <v>19.1</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" t="s">
+        <v>411</v>
+      </c>
+      <c r="G17">
+        <v>17.9</v>
+      </c>
+      <c r="H17">
+        <v>18</v>
+      </c>
+      <c r="I17">
+        <v>18.2</v>
+      </c>
+      <c r="J17">
+        <v>18.2</v>
+      </c>
+      <c r="K17">
+        <v>18.2</v>
+      </c>
+      <c r="L17">
+        <v>18.2</v>
+      </c>
+      <c r="M17">
+        <v>18.3</v>
+      </c>
+      <c r="N17">
+        <v>18.1</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>128</v>
+      </c>
+      <c r="B18" t="s">
+        <v>129</v>
+      </c>
+      <c r="C18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" t="s">
+        <v>412</v>
+      </c>
+      <c r="G18">
+        <v>18.1</v>
+      </c>
+      <c r="H18">
+        <v>18.1</v>
+      </c>
+      <c r="I18">
+        <v>19</v>
+      </c>
+      <c r="J18">
+        <v>19.1</v>
+      </c>
+      <c r="K18">
+        <v>19</v>
+      </c>
+      <c r="L18">
+        <v>19.2</v>
+      </c>
+      <c r="M18">
+        <v>17.8</v>
+      </c>
+      <c r="N18">
+        <v>18.6</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" t="s">
+        <v>413</v>
+      </c>
+      <c r="G19">
+        <v>14.3</v>
+      </c>
+      <c r="H19">
+        <v>13.4</v>
+      </c>
+      <c r="I19">
+        <v>13.4</v>
+      </c>
+      <c r="J19">
+        <v>13.8</v>
+      </c>
+      <c r="K19">
+        <v>13.4</v>
+      </c>
+      <c r="L19">
+        <v>13.4</v>
+      </c>
+      <c r="M19">
+        <v>13.6</v>
+      </c>
+      <c r="N19" s="21">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" t="s">
+        <v>113</v>
+      </c>
+      <c r="D20" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" t="s">
+        <v>114</v>
+      </c>
+      <c r="F20" t="s">
+        <v>404</v>
+      </c>
+      <c r="G20">
+        <v>23.3</v>
+      </c>
+      <c r="H20">
+        <v>23.3</v>
+      </c>
+      <c r="I20">
+        <v>23.3</v>
+      </c>
+      <c r="J20">
+        <v>23.3</v>
+      </c>
+      <c r="K20">
+        <v>23.3</v>
+      </c>
+      <c r="L20">
+        <v>23.3</v>
+      </c>
+      <c r="M20">
+        <v>23.3</v>
+      </c>
+      <c r="N20" s="20">
+        <v>23.3</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>127</v>
+      </c>
+      <c r="B21" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" t="s">
+        <v>111</v>
+      </c>
+      <c r="E21" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" t="s">
+        <v>414</v>
+      </c>
+      <c r="G21">
+        <v>24</v>
+      </c>
+      <c r="H21">
+        <v>24</v>
+      </c>
+      <c r="I21">
+        <v>24</v>
+      </c>
+      <c r="J21">
+        <v>24</v>
+      </c>
+      <c r="K21">
+        <v>24</v>
+      </c>
+      <c r="L21">
+        <v>24</v>
+      </c>
+      <c r="M21">
+        <v>24</v>
+      </c>
+      <c r="N21" s="20">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" t="s">
+        <v>124</v>
+      </c>
+      <c r="D22" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" t="s">
+        <v>415</v>
+      </c>
+      <c r="G22">
+        <v>22.7</v>
+      </c>
+      <c r="H22">
+        <v>22.7</v>
+      </c>
+      <c r="I22">
+        <v>22.7</v>
+      </c>
+      <c r="J22">
+        <v>22.7</v>
+      </c>
+      <c r="K22">
+        <v>22.7</v>
+      </c>
+      <c r="L22">
+        <v>22.7</v>
+      </c>
+      <c r="M22">
+        <v>22.7</v>
+      </c>
+      <c r="N22" s="20">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" t="s">
+        <v>416</v>
+      </c>
+      <c r="G23">
+        <v>22.9</v>
+      </c>
+      <c r="H23">
+        <v>22.9</v>
+      </c>
+      <c r="I23">
+        <v>22.9</v>
+      </c>
+      <c r="J23">
+        <v>22.9</v>
+      </c>
+      <c r="K23">
+        <v>22.9</v>
+      </c>
+      <c r="L23">
+        <v>22.9</v>
+      </c>
+      <c r="M23">
+        <v>22.9</v>
+      </c>
+      <c r="N23" s="20">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" t="s">
+        <v>116</v>
+      </c>
+      <c r="D24" t="s">
+        <v>111</v>
+      </c>
+      <c r="E24" t="s">
+        <v>114</v>
+      </c>
+      <c r="F24" t="s">
+        <v>417</v>
+      </c>
+      <c r="G24">
+        <v>24.2</v>
+      </c>
+      <c r="H24">
+        <v>24.1</v>
+      </c>
+      <c r="I24">
+        <v>24.1</v>
+      </c>
+      <c r="J24">
+        <v>24.1</v>
+      </c>
+      <c r="K24">
+        <v>24.1</v>
+      </c>
+      <c r="L24">
+        <v>24.1</v>
+      </c>
+      <c r="M24">
+        <v>24.1</v>
+      </c>
+      <c r="N24" s="20">
+        <v>24.1</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" t="s">
+        <v>116</v>
+      </c>
+      <c r="C25" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F25" t="s">
+        <v>418</v>
+      </c>
+      <c r="G25">
+        <v>25.5</v>
+      </c>
+      <c r="H25">
+        <v>25.5</v>
+      </c>
+      <c r="I25">
+        <v>25.5</v>
+      </c>
+      <c r="J25">
+        <v>25.5</v>
+      </c>
+      <c r="K25">
+        <v>25.5</v>
+      </c>
+      <c r="L25">
+        <v>25.5</v>
+      </c>
+      <c r="M25">
+        <v>25.5</v>
+      </c>
+      <c r="N25" s="20">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" t="s">
+        <v>88</v>
+      </c>
+      <c r="E26" t="s">
+        <v>91</v>
+      </c>
+      <c r="F26" t="s">
+        <v>419</v>
+      </c>
+      <c r="G26">
+        <v>8.6</v>
+      </c>
+      <c r="H26">
+        <v>8.2</v>
+      </c>
+      <c r="I26">
+        <v>8.2</v>
+      </c>
+      <c r="J26">
+        <v>8</v>
+      </c>
+      <c r="K26">
+        <v>8.3</v>
+      </c>
+      <c r="L26">
+        <v>8</v>
+      </c>
+      <c r="M26">
+        <v>8.1</v>
+      </c>
+      <c r="N26" s="21">
+        <v>8.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>